<commit_message>
Add validated loan outcome construction
</commit_message>
<xml_diff>
--- a/docs/eit/risk_control_matrix.xlsx
+++ b/docs/eit/risk_control_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub Projects\freddie-mac-credit-risk\docs\eit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E862C29-47B9-420C-967F-9AEE368DE594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EAD5BA-CA51-4A5E-B343-6DE7B4FFE69F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="18648" windowHeight="11784" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -385,12 +385,6 @@
     <t>Recalculate outcomes independently for selected loans and reconcile event dates and statuses to the production logic.</t>
   </si>
   <si>
-    <t>Testing workpaper — planned</t>
-  </si>
-  <si>
-    <t>Perform after the chunked loan-level outcome table is created.</t>
-  </si>
-  <si>
     <t>EIT-14</t>
   </si>
   <si>
@@ -643,10 +637,16 @@
     <t>Pass — no invalid delinquency statuses, modification flags, zero-balance codes, tested date formats, or Current Actual UPB values were identified.</t>
   </si>
   <si>
-    <t>02_performance_audit.ipynb — reporting-period coverage by vintage</t>
-  </si>
-  <si>
-    <t>Performance coverage through 202603 was confirmed. Loan-level outcome construction and outcome-window eligibility testing remain to be completed.</t>
+    <t>03_outcome_construction.ipynb — full-population outcome eligibility and censoring tests; 05_outcome_testing_workpaper.md</t>
+  </si>
+  <si>
+    <t>Pass — 12-, 24-, and 36-month outcome windows were constructed for 200,000 loans. Eligibility and censoring classifications reconciled without exception.</t>
+  </si>
+  <si>
+    <t>03_outcome_construction.ipynb — independent 120-loan outcome recalculation; 05_outcome_testing_workpaper.md</t>
+  </si>
+  <si>
+    <t>Pass — 120 stratified sample loans and 6,791 raw performance records were independently recalculated. All outcomes, observation windows, eligibility classifications, and censoring classifications matched.</t>
   </si>
 </sst>
 </file>
@@ -1105,28 +1105,59 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1136,59 +1167,28 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1508,66 +1508,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="26"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="48"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="27"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="29"/>
+      <c r="A4" s="49"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
+      <c r="J4" s="50"/>
+      <c r="K4" s="50"/>
+      <c r="L4" s="51"/>
     </row>
     <row r="6" spans="1:12" ht="42" customHeight="1">
       <c r="A6" s="1" t="s">
@@ -1636,13 +1636,13 @@
         <v>23</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="94.05" customHeight="1">
@@ -1750,13 +1750,13 @@
         <v>50</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="94.05" customHeight="1">
@@ -1940,13 +1940,13 @@
         <v>89</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="94.05" customHeight="1">
@@ -1978,13 +1978,13 @@
         <v>95</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="94.05" customHeight="1">
@@ -2016,13 +2016,13 @@
         <v>100</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="94.05" customHeight="1">
@@ -2054,13 +2054,13 @@
         <v>107</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="94.05" customHeight="1">
@@ -2092,89 +2092,89 @@
         <v>115</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="94.05" customHeight="1">
       <c r="A20" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="G20" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="H20" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="I20" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="J20" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>126</v>
       </c>
       <c r="K20" s="6" t="s">
         <v>90</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="94.05" customHeight="1">
       <c r="A21" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>132</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>113</v>
       </c>
       <c r="H21" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="J21" s="4" t="s">
         <v>133</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="K21" s="7" t="s">
         <v>90</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2229,28 +2229,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="30" t="s">
-        <v>137</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
+      <c r="A1" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="1:8" ht="14.4">
-      <c r="A2" s="31" t="s">
-        <v>138</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
+      <c r="A2" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
     </row>
     <row r="3" spans="1:8" ht="14.4">
       <c r="A3" s="8"/>
@@ -2263,22 +2263,22 @@
       <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" ht="14.4">
-      <c r="A4" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="B4" s="32"/>
+      <c r="A4" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="43"/>
       <c r="C4" s="8"/>
-      <c r="D4" s="32" t="s">
-        <v>140</v>
-      </c>
-      <c r="E4" s="32"/>
+      <c r="D4" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="E4" s="43"/>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" ht="14.4">
       <c r="A5" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B5" s="10">
         <f>COUNTA('Risk-Control Matrix'!$A$7:$A$21)</f>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="B6" s="10">
         <f>COUNTIF('Risk-Control Matrix'!$K$7:$K$21,"Complete")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="9" t="s">
@@ -2318,15 +2318,15 @@
     </row>
     <row r="7" spans="1:8" ht="14.4">
       <c r="A7" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIF('Risk-Control Matrix'!$K$7:$K$21,"Partially Complete")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E7" s="10">
         <f>COUNTIF('Risk-Control Matrix'!$B$7:$B$21,"Low")</f>
@@ -2338,11 +2338,11 @@
     </row>
     <row r="8" spans="1:8" ht="14.4">
       <c r="A8" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIF('Risk-Control Matrix'!$K$7:$K$21,"Not Started")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -2353,11 +2353,11 @@
     </row>
     <row r="9" spans="1:8" ht="14.4">
       <c r="A9" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B9" s="11">
         <f>B6/B5</f>
-        <v>0.73333333333333328</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -2377,48 +2377,48 @@
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="14.4">
-      <c r="A11" s="33" t="s">
-        <v>146</v>
-      </c>
-      <c r="B11" s="33"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="33"/>
+      <c r="A11" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
     </row>
     <row r="12" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A12" s="34" t="s">
-        <v>147</v>
-      </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="36"/>
+      <c r="A12" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="24"/>
     </row>
     <row r="13" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="39"/>
+      <c r="A13" s="25"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="27"/>
     </row>
     <row r="14" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A14" s="40"/>
-      <c r="B14" s="41"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="42"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
     </row>
     <row r="15" spans="1:8" ht="14.4">
       <c r="A15" s="8"/>
@@ -2431,58 +2431,58 @@
       <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8" ht="14.4">
-      <c r="A16" s="33" t="s">
-        <v>148</v>
-      </c>
-      <c r="B16" s="33"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
+      <c r="A16" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
     </row>
     <row r="17" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A17" s="43" t="s">
-        <v>149</v>
-      </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="45"/>
+      <c r="A17" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="34"/>
     </row>
     <row r="18" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A18" s="46"/>
-      <c r="B18" s="47"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="47"/>
-      <c r="E18" s="47"/>
-      <c r="F18" s="47"/>
-      <c r="G18" s="47"/>
-      <c r="H18" s="48"/>
+      <c r="A18" s="35"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="37"/>
     </row>
     <row r="19" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A19" s="46"/>
-      <c r="B19" s="47"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="48"/>
+      <c r="A19" s="35"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="37"/>
     </row>
     <row r="20" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A20" s="49"/>
-      <c r="B20" s="50"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="50"/>
-      <c r="F20" s="50"/>
-      <c r="G20" s="50"/>
-      <c r="H20" s="51"/>
+      <c r="A20" s="38"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2512,7 +2512,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21">
       <c r="A1" s="52" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -2520,30 +2520,30 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="D3" s="12" t="s">
         <v>152</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55.95" customHeight="1">
       <c r="A4" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="D4" s="13" t="s">
         <v>156</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55.95" customHeight="1">
@@ -2554,10 +2554,10 @@
         <v>34</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55.95" customHeight="1">
@@ -2568,10 +2568,10 @@
         <v>24</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="55.95" customHeight="1">
@@ -2582,10 +2582,10 @@
         <v>90</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55.95" customHeight="1">
@@ -2593,13 +2593,13 @@
         <v>9</v>
       </c>
       <c r="B8" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="D8" s="14" t="s">
         <v>165</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="55.95" customHeight="1">
@@ -2607,97 +2607,97 @@
         <v>9</v>
       </c>
       <c r="B9" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" s="14" t="s">
         <v>168</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="55.95" customHeight="1">
       <c r="A10" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="D10" s="14" t="s">
         <v>172</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="55.95" customHeight="1">
       <c r="A11" s="18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B11" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="D11" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="55.95" customHeight="1">
       <c r="A12" s="18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B12" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="D12" s="14" t="s">
         <v>178</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="55.95" customHeight="1">
       <c r="A13" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="D13" s="14" t="s">
         <v>182</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="55.95" customHeight="1">
       <c r="A14" s="18" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B14" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="D14" s="14" t="s">
         <v>185</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="55.95" customHeight="1">
       <c r="A15" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="D15" s="15" t="s">
         <v>189</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add feature engineering and leakage controls
</commit_message>
<xml_diff>
--- a/docs/eit/risk_control_matrix.xlsx
+++ b/docs/eit/risk_control_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub Projects\freddie-mac-credit-risk\docs\eit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EAD5BA-CA51-4A5E-B343-6DE7B4FFE69F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E4AFA8-F03E-4C56-8644-5DF2A226787F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="18648" windowHeight="11784" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -409,12 +409,6 @@
     <t>Review every predictor's availability date and validate the 2015–2016 training and 2017 testing design.</t>
   </si>
   <si>
-    <t>Model methodology workpaper — planned</t>
-  </si>
-  <si>
-    <t>Complete before fitting the logistic-regression PD model.</t>
-  </si>
-  <si>
     <t>EIT-15</t>
   </si>
   <si>
@@ -647,6 +641,12 @@
   </si>
   <si>
     <t>Pass — 120 stratified sample loans and 6,791 raw performance records were independently recalculated. All outcomes, observation windows, eligibility classifications, and censoring classifications matched.</t>
+  </si>
+  <si>
+    <t>04_feature_engineering.ipynb — time-based split, feature manifest, stability and leakage controls; 06_feature_leakage_workpaper.md</t>
+  </si>
+  <si>
+    <t>Feature selection, 2015–2016 development and 2017 test separation, categorical stability, and predictor-level leakage controls passed. Final model-pipeline fitting and methodology review remain.</t>
   </si>
 </sst>
 </file>
@@ -1636,13 +1636,13 @@
         <v>23</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="94.05" customHeight="1">
@@ -1750,13 +1750,13 @@
         <v>50</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="94.05" customHeight="1">
@@ -1940,13 +1940,13 @@
         <v>89</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="94.05" customHeight="1">
@@ -1978,13 +1978,13 @@
         <v>95</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="94.05" customHeight="1">
@@ -2016,13 +2016,13 @@
         <v>100</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="94.05" customHeight="1">
@@ -2054,13 +2054,13 @@
         <v>107</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="94.05" customHeight="1">
@@ -2092,13 +2092,13 @@
         <v>115</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K19" s="6" t="s">
         <v>34</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="94.05" customHeight="1">
@@ -2130,51 +2130,51 @@
         <v>123</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>124</v>
+        <v>202</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>125</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="94.05" customHeight="1">
       <c r="A21" s="7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>130</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>113</v>
       </c>
       <c r="H21" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="J21" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>133</v>
       </c>
       <c r="K21" s="7" t="s">
         <v>90</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2230,7 +2230,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
@@ -2242,7 +2242,7 @@
     </row>
     <row r="2" spans="1:8" ht="14.4">
       <c r="A2" s="42" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B2" s="42"/>
       <c r="C2" s="42"/>
@@ -2264,12 +2264,12 @@
     </row>
     <row r="4" spans="1:8" ht="14.4">
       <c r="A4" s="43" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B4" s="43"/>
       <c r="C4" s="8"/>
       <c r="D4" s="43" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E4" s="43"/>
       <c r="F4" s="8"/>
@@ -2278,7 +2278,7 @@
     </row>
     <row r="5" spans="1:8" ht="14.4">
       <c r="A5" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B5" s="10">
         <f>COUNTA('Risk-Control Matrix'!$A$7:$A$21)</f>
@@ -2318,15 +2318,15 @@
     </row>
     <row r="7" spans="1:8" ht="14.4">
       <c r="A7" s="9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIF('Risk-Control Matrix'!$K$7:$K$21,"Partially Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E7" s="10">
         <f>COUNTIF('Risk-Control Matrix'!$B$7:$B$21,"Low")</f>
@@ -2338,11 +2338,11 @@
     </row>
     <row r="8" spans="1:8" ht="14.4">
       <c r="A8" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIF('Risk-Control Matrix'!$K$7:$K$21,"Not Started")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -2353,7 +2353,7 @@
     </row>
     <row r="9" spans="1:8" ht="14.4">
       <c r="A9" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B9" s="11">
         <f>B6/B5</f>
@@ -2378,7 +2378,7 @@
     </row>
     <row r="11" spans="1:8" ht="14.4">
       <c r="A11" s="31" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B11" s="31"/>
       <c r="C11" s="31"/>
@@ -2390,7 +2390,7 @@
     </row>
     <row r="12" spans="1:8" ht="28.05" customHeight="1">
       <c r="A12" s="22" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="23"/>
@@ -2432,7 +2432,7 @@
     </row>
     <row r="16" spans="1:8" ht="14.4">
       <c r="A16" s="31" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B16" s="31"/>
       <c r="C16" s="31"/>
@@ -2444,7 +2444,7 @@
     </row>
     <row r="17" spans="1:8" ht="28.05" customHeight="1">
       <c r="A17" s="32" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B17" s="33"/>
       <c r="C17" s="33"/>
@@ -2512,7 +2512,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21">
       <c r="A1" s="52" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -2520,30 +2520,30 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="D3" s="12" t="s">
         <v>150</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="55.95" customHeight="1">
       <c r="A4" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="D4" s="13" t="s">
         <v>154</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55.95" customHeight="1">
@@ -2554,10 +2554,10 @@
         <v>34</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55.95" customHeight="1">
@@ -2568,10 +2568,10 @@
         <v>24</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="55.95" customHeight="1">
@@ -2582,10 +2582,10 @@
         <v>90</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55.95" customHeight="1">
@@ -2593,13 +2593,13 @@
         <v>9</v>
       </c>
       <c r="B8" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D8" s="14" t="s">
         <v>163</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="55.95" customHeight="1">
@@ -2607,97 +2607,97 @@
         <v>9</v>
       </c>
       <c r="B9" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D9" s="14" t="s">
         <v>166</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="55.95" customHeight="1">
       <c r="A10" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="D10" s="14" t="s">
         <v>170</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="55.95" customHeight="1">
       <c r="A11" s="18" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B11" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" s="14" t="s">
         <v>173</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="55.95" customHeight="1">
       <c r="A12" s="18" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B12" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="D12" s="14" t="s">
         <v>176</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="55.95" customHeight="1">
       <c r="A13" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="D13" s="14" t="s">
         <v>180</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="55.95" customHeight="1">
       <c r="A14" s="18" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B14" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="D14" s="14" t="s">
         <v>183</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="55.95" customHeight="1">
       <c r="A15" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="D15" s="15" t="s">
         <v>187</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>